<commit_message>
feat: Camtrack SFTP, per-recipient emails, active/ folder for Wialon notifications
</commit_message>
<xml_diff>
--- a/downloads/Livraison 01-04-2026.1_updated-with-order.xlsx
+++ b/downloads/Livraison 01-04-2026.1_updated-with-order.xlsx
@@ -1,12 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="27810" windowHeight="12450"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Routing and scheduling_2" state="visible" r:id="rId4"/>
+    <sheet name="Routing and scheduling_2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -91,7 +94,7 @@
     <t>01.04.2026 06:00</t>
   </si>
   <si>
-    <t>Mamy.RABARIARINJATOVO@galana.mg</t>
+    <t>alanic.nguetsa@camtrack.net</t>
   </si>
   <si>
     <t>DEPOT RAFFINERIE TERMINAL</t>
@@ -694,21 +697,175 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="21">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <family val="2"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -718,10 +875,197 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB0C4DE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -730,33 +1074,328 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="48" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="60% - Accent6" xfId="1" builtinId="52"/>
+    <cellStyle name="40% - Accent6" xfId="2" builtinId="51"/>
+    <cellStyle name="60% - Accent5" xfId="3" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="4" builtinId="49"/>
+    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
+    <cellStyle name="20% - Accent5" xfId="6" builtinId="46"/>
+    <cellStyle name="60% - Accent4" xfId="7" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="8" builtinId="45"/>
+    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
+    <cellStyle name="Accent4" xfId="10" builtinId="41"/>
+    <cellStyle name="Linked Cell" xfId="11" builtinId="24"/>
+    <cellStyle name="40% - Accent3" xfId="12" builtinId="39"/>
+    <cellStyle name="60% - Accent2" xfId="13" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="14" builtinId="37"/>
+    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
+    <cellStyle name="20% - Accent2" xfId="16" builtinId="34"/>
+    <cellStyle name="Accent2" xfId="17" builtinId="33"/>
+    <cellStyle name="40% - Accent1" xfId="18" builtinId="31"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
+    <cellStyle name="Accent1" xfId="20" builtinId="29"/>
+    <cellStyle name="Neutral" xfId="21" builtinId="28"/>
+    <cellStyle name="60% - Accent1" xfId="22" builtinId="32"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="20% - Accent4" xfId="24" builtinId="42"/>
+    <cellStyle name="Total" xfId="25" builtinId="25"/>
+    <cellStyle name="Output" xfId="26" builtinId="21"/>
+    <cellStyle name="Currency" xfId="27" builtinId="4"/>
+    <cellStyle name="20% - Accent3" xfId="28" builtinId="38"/>
+    <cellStyle name="Note" xfId="29" builtinId="10"/>
+    <cellStyle name="Input" xfId="30" builtinId="20"/>
+    <cellStyle name="Heading 4" xfId="31" builtinId="19"/>
+    <cellStyle name="Calculation" xfId="32" builtinId="22"/>
+    <cellStyle name="Good" xfId="33" builtinId="26"/>
+    <cellStyle name="Heading 3" xfId="34" builtinId="18"/>
+    <cellStyle name="CExplanatory Text" xfId="35" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="36" builtinId="16"/>
+    <cellStyle name="Comma [0]" xfId="37" builtinId="6"/>
+    <cellStyle name="20% - Accent6" xfId="38" builtinId="50"/>
+    <cellStyle name="Title" xfId="39" builtinId="15"/>
+    <cellStyle name="Currency [0]" xfId="40" builtinId="7"/>
+    <cellStyle name="Warning Text" xfId="41" builtinId="11"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9"/>
+    <cellStyle name="Heading 2" xfId="43" builtinId="17"/>
+    <cellStyle name="Comma" xfId="44" builtinId="3"/>
+    <cellStyle name="Check Cell" xfId="45" builtinId="23"/>
+    <cellStyle name="60% - Accent3" xfId="46" builtinId="40"/>
+    <cellStyle name="Percent" xfId="47" builtinId="5"/>
+    <cellStyle name="Hyperlink" xfId="48" builtinId="8"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1078,31 +1717,31 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S96"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.07" customWidth="1"/>
-    <col min="2" max="2" width="13.21" customWidth="1"/>
-    <col min="3" max="4" width="13.07" customWidth="1"/>
-    <col min="5" max="5" width="13.21" customWidth="1"/>
-    <col min="6" max="7" width="13.07" customWidth="1"/>
-    <col min="8" max="8" width="21.79" customWidth="1"/>
-    <col min="9" max="10" width="13.07" customWidth="1"/>
+    <col min="1" max="1" width="13.0666666666667" customWidth="1"/>
+    <col min="2" max="2" width="13.2133333333333" customWidth="1"/>
+    <col min="3" max="4" width="13.0666666666667" customWidth="1"/>
+    <col min="5" max="5" width="13.2133333333333" customWidth="1"/>
+    <col min="6" max="7" width="13.0666666666667" customWidth="1"/>
+    <col min="8" max="8" width="21.7933333333333" customWidth="1"/>
+    <col min="9" max="10" width="13.0666666666667" customWidth="1"/>
     <col min="11" max="11" width="38.36" customWidth="1"/>
     <col min="12" max="12" width="39.5" customWidth="1"/>
     <col min="13" max="16" width="4.5" customWidth="1"/>
-    <col min="17" max="17" width="13.21" customWidth="1"/>
-    <col min="18" max="18" width="13.07" customWidth="1"/>
-    <col min="19" max="19" width="14.79" customWidth="1"/>
+    <col min="17" max="17" width="13.2133333333333" customWidth="1"/>
+    <col min="18" max="18" width="13.0666666666667" customWidth="1"/>
+    <col min="19" max="19" width="32.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" ht="45" customHeight="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1161,7 +1800,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19">
       <c r="A2">
         <v>33681</v>
       </c>
@@ -1216,11 +1855,11 @@
       <c r="R2" t="s">
         <v>19</v>
       </c>
-      <c r="S2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S2" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
       <c r="A3">
         <v>33681</v>
       </c>
@@ -1275,11 +1914,11 @@
       <c r="R3" t="s">
         <v>19</v>
       </c>
-      <c r="S3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S3" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
       <c r="A4">
         <v>33681</v>
       </c>
@@ -1334,11 +1973,11 @@
       <c r="R4" t="s">
         <v>19</v>
       </c>
-      <c r="S4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S4" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
       <c r="A5">
         <v>33678</v>
       </c>
@@ -1393,11 +2032,11 @@
       <c r="R5" t="s">
         <v>19</v>
       </c>
-      <c r="S5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S5" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
       <c r="A6">
         <v>33678</v>
       </c>
@@ -1452,11 +2091,11 @@
       <c r="R6" t="s">
         <v>19</v>
       </c>
-      <c r="S6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S6" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
       <c r="A7">
         <v>33678</v>
       </c>
@@ -1511,11 +2150,11 @@
       <c r="R7" t="s">
         <v>19</v>
       </c>
-      <c r="S7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
       <c r="A8">
         <v>33678</v>
       </c>
@@ -1570,11 +2209,11 @@
       <c r="R8" t="s">
         <v>19</v>
       </c>
-      <c r="S8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S8" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
       <c r="A9">
         <v>33695</v>
       </c>
@@ -1629,11 +2268,11 @@
       <c r="R9" t="s">
         <v>19</v>
       </c>
-      <c r="S9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
       <c r="A10">
         <v>33695</v>
       </c>
@@ -1688,11 +2327,11 @@
       <c r="R10" t="s">
         <v>19</v>
       </c>
-      <c r="S10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S10" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19">
       <c r="A11">
         <v>33695</v>
       </c>
@@ -1747,11 +2386,11 @@
       <c r="R11" t="s">
         <v>19</v>
       </c>
-      <c r="S11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19">
       <c r="A12">
         <v>33678</v>
       </c>
@@ -1806,11 +2445,11 @@
       <c r="R12" t="s">
         <v>19</v>
       </c>
-      <c r="S12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19">
       <c r="A13">
         <v>33688</v>
       </c>
@@ -1865,11 +2504,11 @@
       <c r="R13" t="s">
         <v>19</v>
       </c>
-      <c r="S13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S13" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19">
       <c r="A14">
         <v>33678</v>
       </c>
@@ -1924,11 +2563,11 @@
       <c r="R14" t="s">
         <v>19</v>
       </c>
-      <c r="S14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S14" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19">
       <c r="A15">
         <v>33678</v>
       </c>
@@ -1983,11 +2622,11 @@
       <c r="R15" t="s">
         <v>19</v>
       </c>
-      <c r="S15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S15" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19">
       <c r="A16">
         <v>33678</v>
       </c>
@@ -2042,11 +2681,11 @@
       <c r="R16" t="s">
         <v>19</v>
       </c>
-      <c r="S16" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S16" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19">
       <c r="A17">
         <v>33688</v>
       </c>
@@ -2101,11 +2740,11 @@
       <c r="R17" t="s">
         <v>19</v>
       </c>
-      <c r="S17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S17" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19">
       <c r="A18">
         <v>33688</v>
       </c>
@@ -2160,11 +2799,11 @@
       <c r="R18" t="s">
         <v>19</v>
       </c>
-      <c r="S18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S18" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19">
       <c r="A19">
         <v>33687</v>
       </c>
@@ -2219,11 +2858,11 @@
       <c r="R19" t="s">
         <v>19</v>
       </c>
-      <c r="S19" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S19" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19">
       <c r="A20">
         <v>33687</v>
       </c>
@@ -2278,11 +2917,11 @@
       <c r="R20" t="s">
         <v>19</v>
       </c>
-      <c r="S20" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S20" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19">
       <c r="A21">
         <v>33687</v>
       </c>
@@ -2337,11 +2976,11 @@
       <c r="R21" t="s">
         <v>19</v>
       </c>
-      <c r="S21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S21" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19">
       <c r="A22">
         <v>33678</v>
       </c>
@@ -2396,11 +3035,11 @@
       <c r="R22" t="s">
         <v>19</v>
       </c>
-      <c r="S22" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S22" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19">
       <c r="A23">
         <v>33678</v>
       </c>
@@ -2455,11 +3094,11 @@
       <c r="R23" t="s">
         <v>19</v>
       </c>
-      <c r="S23" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S23" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19">
       <c r="A24">
         <v>33678</v>
       </c>
@@ -2514,11 +3153,11 @@
       <c r="R24" t="s">
         <v>19</v>
       </c>
-      <c r="S24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S24" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19">
       <c r="A25">
         <v>33678</v>
       </c>
@@ -2573,11 +3212,11 @@
       <c r="R25" t="s">
         <v>19</v>
       </c>
-      <c r="S25" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S25" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19">
       <c r="A26">
         <v>33678</v>
       </c>
@@ -2632,11 +3271,11 @@
       <c r="R26" t="s">
         <v>19</v>
       </c>
-      <c r="S26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S26" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19">
       <c r="A27">
         <v>33678</v>
       </c>
@@ -2691,11 +3330,11 @@
       <c r="R27" t="s">
         <v>19</v>
       </c>
-      <c r="S27" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S27" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19">
       <c r="A28">
         <v>33678</v>
       </c>
@@ -2750,11 +3389,11 @@
       <c r="R28" t="s">
         <v>19</v>
       </c>
-      <c r="S28" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S28" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19">
       <c r="A29">
         <v>33678</v>
       </c>
@@ -2809,11 +3448,11 @@
       <c r="R29" t="s">
         <v>19</v>
       </c>
-      <c r="S29" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S29" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19">
       <c r="A30">
         <v>33678</v>
       </c>
@@ -2868,11 +3507,11 @@
       <c r="R30" t="s">
         <v>19</v>
       </c>
-      <c r="S30" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S30" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19">
       <c r="A31">
         <v>33678</v>
       </c>
@@ -2927,11 +3566,11 @@
       <c r="R31" t="s">
         <v>19</v>
       </c>
-      <c r="S31" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S31" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19">
       <c r="A32">
         <v>33678</v>
       </c>
@@ -2986,11 +3625,11 @@
       <c r="R32" t="s">
         <v>19</v>
       </c>
-      <c r="S32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S32" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19">
       <c r="A33">
         <v>33678</v>
       </c>
@@ -3045,11 +3684,11 @@
       <c r="R33" t="s">
         <v>19</v>
       </c>
-      <c r="S33" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S33" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19">
       <c r="A34">
         <v>33678</v>
       </c>
@@ -3104,11 +3743,11 @@
       <c r="R34" t="s">
         <v>19</v>
       </c>
-      <c r="S34" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S34" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19">
       <c r="A35">
         <v>33678</v>
       </c>
@@ -3163,11 +3802,11 @@
       <c r="R35" t="s">
         <v>19</v>
       </c>
-      <c r="S35" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S35" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19">
       <c r="A36">
         <v>33678</v>
       </c>
@@ -3222,11 +3861,11 @@
       <c r="R36" t="s">
         <v>19</v>
       </c>
-      <c r="S36" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S36" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19">
       <c r="A37">
         <v>33678</v>
       </c>
@@ -3281,11 +3920,11 @@
       <c r="R37" t="s">
         <v>19</v>
       </c>
-      <c r="S37" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S37" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19">
       <c r="A38">
         <v>33678</v>
       </c>
@@ -3340,11 +3979,11 @@
       <c r="R38" t="s">
         <v>19</v>
       </c>
-      <c r="S38" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S38" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19">
       <c r="A39">
         <v>33678</v>
       </c>
@@ -3399,11 +4038,11 @@
       <c r="R39" t="s">
         <v>19</v>
       </c>
-      <c r="S39" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S39" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19">
       <c r="A40">
         <v>33678</v>
       </c>
@@ -3458,11 +4097,11 @@
       <c r="R40" t="s">
         <v>19</v>
       </c>
-      <c r="S40" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S40" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19">
       <c r="A41">
         <v>33702</v>
       </c>
@@ -3517,11 +4156,11 @@
       <c r="R41" t="s">
         <v>19</v>
       </c>
-      <c r="S41" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S41" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19">
       <c r="A42">
         <v>33702</v>
       </c>
@@ -3576,11 +4215,11 @@
       <c r="R42" t="s">
         <v>19</v>
       </c>
-      <c r="S42" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S42" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19">
       <c r="A43">
         <v>33702</v>
       </c>
@@ -3635,11 +4274,11 @@
       <c r="R43" t="s">
         <v>19</v>
       </c>
-      <c r="S43" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S43" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19">
       <c r="A44">
         <v>33702</v>
       </c>
@@ -3694,11 +4333,11 @@
       <c r="R44" t="s">
         <v>19</v>
       </c>
-      <c r="S44" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S44" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19">
       <c r="A45">
         <v>33702</v>
       </c>
@@ -3753,11 +4392,11 @@
       <c r="R45" t="s">
         <v>19</v>
       </c>
-      <c r="S45" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S45" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19">
       <c r="A46">
         <v>33702</v>
       </c>
@@ -3812,11 +4451,11 @@
       <c r="R46" t="s">
         <v>19</v>
       </c>
-      <c r="S46" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S46" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19">
       <c r="A47">
         <v>33693</v>
       </c>
@@ -3871,11 +4510,11 @@
       <c r="R47" t="s">
         <v>19</v>
       </c>
-      <c r="S47" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S47" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19">
       <c r="A48">
         <v>33693</v>
       </c>
@@ -3930,11 +4569,11 @@
       <c r="R48" t="s">
         <v>19</v>
       </c>
-      <c r="S48" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S48" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19">
       <c r="A49">
         <v>33693</v>
       </c>
@@ -3989,11 +4628,11 @@
       <c r="R49" t="s">
         <v>19</v>
       </c>
-      <c r="S49" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S49" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19">
       <c r="A50">
         <v>33693</v>
       </c>
@@ -4048,11 +4687,11 @@
       <c r="R50" t="s">
         <v>19</v>
       </c>
-      <c r="S50" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S50" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19">
       <c r="A51">
         <v>33678</v>
       </c>
@@ -4107,11 +4746,11 @@
       <c r="R51" t="s">
         <v>19</v>
       </c>
-      <c r="S51" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S51" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19">
       <c r="A52">
         <v>33678</v>
       </c>
@@ -4166,11 +4805,11 @@
       <c r="R52" t="s">
         <v>19</v>
       </c>
-      <c r="S52" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S52" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19">
       <c r="A53">
         <v>33678</v>
       </c>
@@ -4225,11 +4864,11 @@
       <c r="R53" t="s">
         <v>19</v>
       </c>
-      <c r="S53" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S53" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19">
       <c r="A54">
         <v>33678</v>
       </c>
@@ -4284,11 +4923,11 @@
       <c r="R54" t="s">
         <v>19</v>
       </c>
-      <c r="S54" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S54" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19">
       <c r="A55">
         <v>33678</v>
       </c>
@@ -4343,11 +4982,11 @@
       <c r="R55" t="s">
         <v>19</v>
       </c>
-      <c r="S55" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S55" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19">
       <c r="A56">
         <v>33678</v>
       </c>
@@ -4402,11 +5041,11 @@
       <c r="R56" t="s">
         <v>19</v>
       </c>
-      <c r="S56" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S56" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19">
       <c r="A57">
         <v>33678</v>
       </c>
@@ -4461,11 +5100,11 @@
       <c r="R57" t="s">
         <v>19</v>
       </c>
-      <c r="S57" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S57" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19">
       <c r="A58">
         <v>33678</v>
       </c>
@@ -4520,11 +5159,11 @@
       <c r="R58" t="s">
         <v>19</v>
       </c>
-      <c r="S58" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S58" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19">
       <c r="A59">
         <v>33678</v>
       </c>
@@ -4579,11 +5218,11 @@
       <c r="R59" t="s">
         <v>19</v>
       </c>
-      <c r="S59" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S59" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19">
       <c r="A60">
         <v>33678</v>
       </c>
@@ -4638,11 +5277,11 @@
       <c r="R60" t="s">
         <v>19</v>
       </c>
-      <c r="S60" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S60" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19">
       <c r="A61">
         <v>33678</v>
       </c>
@@ -4697,11 +5336,11 @@
       <c r="R61" t="s">
         <v>19</v>
       </c>
-      <c r="S61" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S61" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19">
       <c r="A62">
         <v>33678</v>
       </c>
@@ -4756,11 +5395,11 @@
       <c r="R62" t="s">
         <v>19</v>
       </c>
-      <c r="S62" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S62" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="63" spans="1:19">
       <c r="A63">
         <v>33690</v>
       </c>
@@ -4815,11 +5454,11 @@
       <c r="R63" t="s">
         <v>19</v>
       </c>
-      <c r="S63" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S63" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19">
       <c r="A64">
         <v>33690</v>
       </c>
@@ -4874,11 +5513,11 @@
       <c r="R64" t="s">
         <v>19</v>
       </c>
-      <c r="S64" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S64" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19">
       <c r="A65">
         <v>33690</v>
       </c>
@@ -4933,11 +5572,11 @@
       <c r="R65" t="s">
         <v>19</v>
       </c>
-      <c r="S65" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S65" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19">
       <c r="A66">
         <v>33690</v>
       </c>
@@ -4992,11 +5631,11 @@
       <c r="R66" t="s">
         <v>19</v>
       </c>
-      <c r="S66" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S66" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19">
       <c r="A67">
         <v>33690</v>
       </c>
@@ -5051,11 +5690,11 @@
       <c r="R67" t="s">
         <v>19</v>
       </c>
-      <c r="S67" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S67" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19">
       <c r="A68">
         <v>33678</v>
       </c>
@@ -5110,11 +5749,11 @@
       <c r="R68" t="s">
         <v>19</v>
       </c>
-      <c r="S68" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S68" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="69" spans="1:19">
       <c r="A69">
         <v>33678</v>
       </c>
@@ -5169,11 +5808,11 @@
       <c r="R69" t="s">
         <v>19</v>
       </c>
-      <c r="S69" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S69" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19">
       <c r="A70">
         <v>33678</v>
       </c>
@@ -5228,11 +5867,11 @@
       <c r="R70" t="s">
         <v>19</v>
       </c>
-      <c r="S70" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S70" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19">
       <c r="A71">
         <v>33678</v>
       </c>
@@ -5287,11 +5926,11 @@
       <c r="R71" t="s">
         <v>19</v>
       </c>
-      <c r="S71" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S71" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="72" spans="1:19">
       <c r="A72">
         <v>33678</v>
       </c>
@@ -5346,11 +5985,11 @@
       <c r="R72" t="s">
         <v>19</v>
       </c>
-      <c r="S72" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S72" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="73" spans="1:19">
       <c r="A73">
         <v>33678</v>
       </c>
@@ -5405,11 +6044,11 @@
       <c r="R73" t="s">
         <v>19</v>
       </c>
-      <c r="S73" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S73" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="74" spans="1:19">
       <c r="A74">
         <v>33678</v>
       </c>
@@ -5464,11 +6103,11 @@
       <c r="R74" t="s">
         <v>19</v>
       </c>
-      <c r="S74" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S74" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:19">
       <c r="A75">
         <v>33685</v>
       </c>
@@ -5523,11 +6162,11 @@
       <c r="R75" t="s">
         <v>19</v>
       </c>
-      <c r="S75" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S75" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="76" spans="1:19">
       <c r="A76">
         <v>33692</v>
       </c>
@@ -5582,11 +6221,11 @@
       <c r="R76" t="s">
         <v>19</v>
       </c>
-      <c r="S76" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S76" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19">
       <c r="A77">
         <v>33685</v>
       </c>
@@ -5641,11 +6280,11 @@
       <c r="R77" t="s">
         <v>19</v>
       </c>
-      <c r="S77" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S77" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19">
       <c r="A78">
         <v>33685</v>
       </c>
@@ -5700,11 +6339,11 @@
       <c r="R78" t="s">
         <v>19</v>
       </c>
-      <c r="S78" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S78" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="79" spans="1:19">
       <c r="A79">
         <v>33692</v>
       </c>
@@ -5759,11 +6398,11 @@
       <c r="R79" t="s">
         <v>19</v>
       </c>
-      <c r="S79" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S79" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19">
       <c r="A80">
         <v>33686</v>
       </c>
@@ -5818,11 +6457,11 @@
       <c r="R80" t="s">
         <v>19</v>
       </c>
-      <c r="S80" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S80" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19">
       <c r="A81">
         <v>33686</v>
       </c>
@@ -5877,11 +6516,11 @@
       <c r="R81" t="s">
         <v>19</v>
       </c>
-      <c r="S81" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S81" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="82" spans="1:19">
       <c r="A82">
         <v>33686</v>
       </c>
@@ -5936,11 +6575,11 @@
       <c r="R82" t="s">
         <v>19</v>
       </c>
-      <c r="S82" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S82" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19">
       <c r="A83">
         <v>33681</v>
       </c>
@@ -5995,11 +6634,11 @@
       <c r="R83" t="s">
         <v>19</v>
       </c>
-      <c r="S83" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S83" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84" spans="1:19">
       <c r="A84">
         <v>33681</v>
       </c>
@@ -6054,11 +6693,11 @@
       <c r="R84" t="s">
         <v>19</v>
       </c>
-      <c r="S84" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S84" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="85" spans="1:19">
       <c r="A85">
         <v>33681</v>
       </c>
@@ -6113,11 +6752,11 @@
       <c r="R85" t="s">
         <v>19</v>
       </c>
-      <c r="S85" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S85" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19">
       <c r="A86">
         <v>33681</v>
       </c>
@@ -6172,11 +6811,11 @@
       <c r="R86" t="s">
         <v>19</v>
       </c>
-      <c r="S86" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S86" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19">
       <c r="A87">
         <v>33676</v>
       </c>
@@ -6231,11 +6870,11 @@
       <c r="R87" t="s">
         <v>19</v>
       </c>
-      <c r="S87" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S87" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:19">
       <c r="A88">
         <v>33700</v>
       </c>
@@ -6290,11 +6929,11 @@
       <c r="R88" t="s">
         <v>19</v>
       </c>
-      <c r="S88" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S88" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19">
       <c r="A89">
         <v>33676</v>
       </c>
@@ -6349,11 +6988,11 @@
       <c r="R89" t="s">
         <v>19</v>
       </c>
-      <c r="S89" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S89" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="90" spans="1:19">
       <c r="A90">
         <v>33676</v>
       </c>
@@ -6408,11 +7047,11 @@
       <c r="R90" t="s">
         <v>19</v>
       </c>
-      <c r="S90" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S90" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19">
       <c r="A91">
         <v>33700</v>
       </c>
@@ -6467,11 +7106,11 @@
       <c r="R91" t="s">
         <v>19</v>
       </c>
-      <c r="S91" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S91" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19">
       <c r="A92">
         <v>33699</v>
       </c>
@@ -6526,11 +7165,11 @@
       <c r="R92" t="s">
         <v>19</v>
       </c>
-      <c r="S92" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S92" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="93" spans="1:19">
       <c r="A93">
         <v>33699</v>
       </c>
@@ -6585,11 +7224,11 @@
       <c r="R93" t="s">
         <v>19</v>
       </c>
-      <c r="S93" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S93" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="94" spans="1:19">
       <c r="A94">
         <v>33699</v>
       </c>
@@ -6644,11 +7283,11 @@
       <c r="R94" t="s">
         <v>19</v>
       </c>
-      <c r="S94" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S94" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="95" spans="1:19">
       <c r="A95" t="s">
         <v>19</v>
       </c>
@@ -6707,7 +7346,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19">
       <c r="A96" t="s">
         <v>19</v>
       </c>
@@ -6767,7 +7406,103 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="S7" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S2" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S3" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S4" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S5" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S6" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S8" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S9" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S10" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S11" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S12" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S13" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S14" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S15" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S16" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S17" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S18" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S19" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S20" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S21" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S22" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S23" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S24" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S25" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S26" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S27" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S28" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S29" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S30" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S31" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S32" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S33" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S34" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S35" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S36" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S37" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S38" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S39" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S40" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S41" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S42" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S43" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S44" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S45" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S46" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S47" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S48" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S49" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S50" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S51" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S52" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S53" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S54" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S55" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S56" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S57" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S58" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S59" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S60" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S61" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S62" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S63" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S64" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S65" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S66" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S67" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S68" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S69" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S70" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S71" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S72" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S73" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S74" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S75" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S76" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S77" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S78" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S79" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S80" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S81" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S82" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S83" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S84" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S85" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S86" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S87" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S88" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S89" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S90" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S91" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S92" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S93" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+    <hyperlink ref="S94" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updates new processes for the report
</commit_message>
<xml_diff>
--- a/downloads/Livraison 01-04-2026.1_updated-with-order.xlsx
+++ b/downloads/Livraison 01-04-2026.1_updated-with-order.xlsx
@@ -1,15 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="27810" windowHeight="12450"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Routing and scheduling_2" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Routing and scheduling_2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -94,7 +91,7 @@
     <t>01.04.2026 06:00</t>
   </si>
   <si>
-    <t>alanic.nguetsa@camtrack.net</t>
+    <t>Mamy.RABARIARINJATOVO@galana.mg</t>
   </si>
   <si>
     <t>DEPOT RAFFINERIE TERMINAL</t>
@@ -697,175 +694,21 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -875,197 +718,10 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB0C4DE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1074,328 +730,33 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="48" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="60% - Accent6" xfId="1" builtinId="52"/>
-    <cellStyle name="40% - Accent6" xfId="2" builtinId="51"/>
-    <cellStyle name="60% - Accent5" xfId="3" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="4" builtinId="49"/>
-    <cellStyle name="40% - Accent5" xfId="5" builtinId="47"/>
-    <cellStyle name="20% - Accent5" xfId="6" builtinId="46"/>
-    <cellStyle name="60% - Accent4" xfId="7" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="8" builtinId="45"/>
-    <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
-    <cellStyle name="Accent4" xfId="10" builtinId="41"/>
-    <cellStyle name="Linked Cell" xfId="11" builtinId="24"/>
-    <cellStyle name="40% - Accent3" xfId="12" builtinId="39"/>
-    <cellStyle name="60% - Accent2" xfId="13" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="14" builtinId="37"/>
-    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
-    <cellStyle name="20% - Accent2" xfId="16" builtinId="34"/>
-    <cellStyle name="Accent2" xfId="17" builtinId="33"/>
-    <cellStyle name="40% - Accent1" xfId="18" builtinId="31"/>
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30"/>
-    <cellStyle name="Accent1" xfId="20" builtinId="29"/>
-    <cellStyle name="Neutral" xfId="21" builtinId="28"/>
-    <cellStyle name="60% - Accent1" xfId="22" builtinId="32"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="20% - Accent4" xfId="24" builtinId="42"/>
-    <cellStyle name="Total" xfId="25" builtinId="25"/>
-    <cellStyle name="Output" xfId="26" builtinId="21"/>
-    <cellStyle name="Currency" xfId="27" builtinId="4"/>
-    <cellStyle name="20% - Accent3" xfId="28" builtinId="38"/>
-    <cellStyle name="Note" xfId="29" builtinId="10"/>
-    <cellStyle name="Input" xfId="30" builtinId="20"/>
-    <cellStyle name="Heading 4" xfId="31" builtinId="19"/>
-    <cellStyle name="Calculation" xfId="32" builtinId="22"/>
-    <cellStyle name="Good" xfId="33" builtinId="26"/>
-    <cellStyle name="Heading 3" xfId="34" builtinId="18"/>
-    <cellStyle name="CExplanatory Text" xfId="35" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="36" builtinId="16"/>
-    <cellStyle name="Comma [0]" xfId="37" builtinId="6"/>
-    <cellStyle name="20% - Accent6" xfId="38" builtinId="50"/>
-    <cellStyle name="Title" xfId="39" builtinId="15"/>
-    <cellStyle name="Currency [0]" xfId="40" builtinId="7"/>
-    <cellStyle name="Warning Text" xfId="41" builtinId="11"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9"/>
-    <cellStyle name="Heading 2" xfId="43" builtinId="17"/>
-    <cellStyle name="Comma" xfId="44" builtinId="3"/>
-    <cellStyle name="Check Cell" xfId="45" builtinId="23"/>
-    <cellStyle name="60% - Accent3" xfId="46" builtinId="40"/>
-    <cellStyle name="Percent" xfId="47" builtinId="5"/>
-    <cellStyle name="Hyperlink" xfId="48" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1717,31 +1078,31 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S96"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="13.0666666666667" customWidth="1"/>
-    <col min="2" max="2" width="13.2133333333333" customWidth="1"/>
-    <col min="3" max="4" width="13.0666666666667" customWidth="1"/>
-    <col min="5" max="5" width="13.2133333333333" customWidth="1"/>
-    <col min="6" max="7" width="13.0666666666667" customWidth="1"/>
-    <col min="8" max="8" width="21.7933333333333" customWidth="1"/>
-    <col min="9" max="10" width="13.0666666666667" customWidth="1"/>
+    <col min="1" max="1" width="13.07" customWidth="1"/>
+    <col min="2" max="2" width="13.21" customWidth="1"/>
+    <col min="3" max="4" width="13.07" customWidth="1"/>
+    <col min="5" max="5" width="13.21" customWidth="1"/>
+    <col min="6" max="7" width="13.07" customWidth="1"/>
+    <col min="8" max="8" width="21.79" customWidth="1"/>
+    <col min="9" max="10" width="13.07" customWidth="1"/>
     <col min="11" max="11" width="38.36" customWidth="1"/>
     <col min="12" max="12" width="39.5" customWidth="1"/>
     <col min="13" max="16" width="4.5" customWidth="1"/>
-    <col min="17" max="17" width="13.2133333333333" customWidth="1"/>
-    <col min="18" max="18" width="13.0666666666667" customWidth="1"/>
-    <col min="19" max="19" width="32.5" customWidth="1"/>
+    <col min="17" max="17" width="13.21" customWidth="1"/>
+    <col min="18" max="18" width="13.07" customWidth="1"/>
+    <col min="19" max="19" width="14.79" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" spans="1:19">
+    <row r="1" ht="45" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1800,7 +1161,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>33681</v>
       </c>
@@ -1855,11 +1216,11 @@
       <c r="R2" t="s">
         <v>19</v>
       </c>
-      <c r="S2" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19">
+      <c r="S2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>33681</v>
       </c>
@@ -1914,11 +1275,11 @@
       <c r="R3" t="s">
         <v>19</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19">
+      <c r="S3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>33681</v>
       </c>
@@ -1973,11 +1334,11 @@
       <c r="R4" t="s">
         <v>19</v>
       </c>
-      <c r="S4" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19">
+      <c r="S4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>33678</v>
       </c>
@@ -2032,11 +1393,11 @@
       <c r="R5" t="s">
         <v>19</v>
       </c>
-      <c r="S5" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19">
+      <c r="S5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>33678</v>
       </c>
@@ -2091,11 +1452,11 @@
       <c r="R6" t="s">
         <v>19</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19">
+      <c r="S6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>33678</v>
       </c>
@@ -2150,11 +1511,11 @@
       <c r="R7" t="s">
         <v>19</v>
       </c>
-      <c r="S7" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19">
+      <c r="S7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>33678</v>
       </c>
@@ -2209,11 +1570,11 @@
       <c r="R8" t="s">
         <v>19</v>
       </c>
-      <c r="S8" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19">
+      <c r="S8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>33695</v>
       </c>
@@ -2268,11 +1629,11 @@
       <c r="R9" t="s">
         <v>19</v>
       </c>
-      <c r="S9" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19">
+      <c r="S9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>33695</v>
       </c>
@@ -2327,11 +1688,11 @@
       <c r="R10" t="s">
         <v>19</v>
       </c>
-      <c r="S10" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19">
+      <c r="S10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>33695</v>
       </c>
@@ -2386,11 +1747,11 @@
       <c r="R11" t="s">
         <v>19</v>
       </c>
-      <c r="S11" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19">
+      <c r="S11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>33678</v>
       </c>
@@ -2445,11 +1806,11 @@
       <c r="R12" t="s">
         <v>19</v>
       </c>
-      <c r="S12" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19">
+      <c r="S12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>33688</v>
       </c>
@@ -2504,11 +1865,11 @@
       <c r="R13" t="s">
         <v>19</v>
       </c>
-      <c r="S13" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19">
+      <c r="S13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>33678</v>
       </c>
@@ -2563,11 +1924,11 @@
       <c r="R14" t="s">
         <v>19</v>
       </c>
-      <c r="S14" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19">
+      <c r="S14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>33678</v>
       </c>
@@ -2622,11 +1983,11 @@
       <c r="R15" t="s">
         <v>19</v>
       </c>
-      <c r="S15" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19">
+      <c r="S15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>33678</v>
       </c>
@@ -2681,11 +2042,11 @@
       <c r="R16" t="s">
         <v>19</v>
       </c>
-      <c r="S16" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19">
+      <c r="S16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>33688</v>
       </c>
@@ -2740,11 +2101,11 @@
       <c r="R17" t="s">
         <v>19</v>
       </c>
-      <c r="S17" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19">
+      <c r="S17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>33688</v>
       </c>
@@ -2799,11 +2160,11 @@
       <c r="R18" t="s">
         <v>19</v>
       </c>
-      <c r="S18" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19">
+      <c r="S18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>33687</v>
       </c>
@@ -2858,11 +2219,11 @@
       <c r="R19" t="s">
         <v>19</v>
       </c>
-      <c r="S19" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19">
+      <c r="S19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>33687</v>
       </c>
@@ -2917,11 +2278,11 @@
       <c r="R20" t="s">
         <v>19</v>
       </c>
-      <c r="S20" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19">
+      <c r="S20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>33687</v>
       </c>
@@ -2976,11 +2337,11 @@
       <c r="R21" t="s">
         <v>19</v>
       </c>
-      <c r="S21" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19">
+      <c r="S21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>33678</v>
       </c>
@@ -3035,11 +2396,11 @@
       <c r="R22" t="s">
         <v>19</v>
       </c>
-      <c r="S22" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:19">
+      <c r="S22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>33678</v>
       </c>
@@ -3094,11 +2455,11 @@
       <c r="R23" t="s">
         <v>19</v>
       </c>
-      <c r="S23" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19">
+      <c r="S23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>33678</v>
       </c>
@@ -3153,11 +2514,11 @@
       <c r="R24" t="s">
         <v>19</v>
       </c>
-      <c r="S24" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19">
+      <c r="S24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>33678</v>
       </c>
@@ -3212,11 +2573,11 @@
       <c r="R25" t="s">
         <v>19</v>
       </c>
-      <c r="S25" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19">
+      <c r="S25" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>33678</v>
       </c>
@@ -3271,11 +2632,11 @@
       <c r="R26" t="s">
         <v>19</v>
       </c>
-      <c r="S26" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19">
+      <c r="S26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>33678</v>
       </c>
@@ -3330,11 +2691,11 @@
       <c r="R27" t="s">
         <v>19</v>
       </c>
-      <c r="S27" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19">
+      <c r="S27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>33678</v>
       </c>
@@ -3389,11 +2750,11 @@
       <c r="R28" t="s">
         <v>19</v>
       </c>
-      <c r="S28" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19">
+      <c r="S28" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>33678</v>
       </c>
@@ -3448,11 +2809,11 @@
       <c r="R29" t="s">
         <v>19</v>
       </c>
-      <c r="S29" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19">
+      <c r="S29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>33678</v>
       </c>
@@ -3507,11 +2868,11 @@
       <c r="R30" t="s">
         <v>19</v>
       </c>
-      <c r="S30" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19">
+      <c r="S30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>33678</v>
       </c>
@@ -3566,11 +2927,11 @@
       <c r="R31" t="s">
         <v>19</v>
       </c>
-      <c r="S31" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19">
+      <c r="S31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>33678</v>
       </c>
@@ -3625,11 +2986,11 @@
       <c r="R32" t="s">
         <v>19</v>
       </c>
-      <c r="S32" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:19">
+      <c r="S32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>33678</v>
       </c>
@@ -3684,11 +3045,11 @@
       <c r="R33" t="s">
         <v>19</v>
       </c>
-      <c r="S33" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19">
+      <c r="S33" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33678</v>
       </c>
@@ -3743,11 +3104,11 @@
       <c r="R34" t="s">
         <v>19</v>
       </c>
-      <c r="S34" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19">
+      <c r="S34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33678</v>
       </c>
@@ -3802,11 +3163,11 @@
       <c r="R35" t="s">
         <v>19</v>
       </c>
-      <c r="S35" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:19">
+      <c r="S35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>33678</v>
       </c>
@@ -3861,11 +3222,11 @@
       <c r="R36" t="s">
         <v>19</v>
       </c>
-      <c r="S36" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19">
+      <c r="S36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>33678</v>
       </c>
@@ -3920,11 +3281,11 @@
       <c r="R37" t="s">
         <v>19</v>
       </c>
-      <c r="S37" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19">
+      <c r="S37" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>33678</v>
       </c>
@@ -3979,11 +3340,11 @@
       <c r="R38" t="s">
         <v>19</v>
       </c>
-      <c r="S38" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19">
+      <c r="S38" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>33678</v>
       </c>
@@ -4038,11 +3399,11 @@
       <c r="R39" t="s">
         <v>19</v>
       </c>
-      <c r="S39" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="40" spans="1:19">
+      <c r="S39" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>33678</v>
       </c>
@@ -4097,11 +3458,11 @@
       <c r="R40" t="s">
         <v>19</v>
       </c>
-      <c r="S40" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="41" spans="1:19">
+      <c r="S40" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>33702</v>
       </c>
@@ -4156,11 +3517,11 @@
       <c r="R41" t="s">
         <v>19</v>
       </c>
-      <c r="S41" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="1:19">
+      <c r="S41" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>33702</v>
       </c>
@@ -4215,11 +3576,11 @@
       <c r="R42" t="s">
         <v>19</v>
       </c>
-      <c r="S42" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="43" spans="1:19">
+      <c r="S42" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>33702</v>
       </c>
@@ -4274,11 +3635,11 @@
       <c r="R43" t="s">
         <v>19</v>
       </c>
-      <c r="S43" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="44" spans="1:19">
+      <c r="S43" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>33702</v>
       </c>
@@ -4333,11 +3694,11 @@
       <c r="R44" t="s">
         <v>19</v>
       </c>
-      <c r="S44" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="45" spans="1:19">
+      <c r="S44" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>33702</v>
       </c>
@@ -4392,11 +3753,11 @@
       <c r="R45" t="s">
         <v>19</v>
       </c>
-      <c r="S45" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="46" spans="1:19">
+      <c r="S45" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>33702</v>
       </c>
@@ -4451,11 +3812,11 @@
       <c r="R46" t="s">
         <v>19</v>
       </c>
-      <c r="S46" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="47" spans="1:19">
+      <c r="S46" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>33693</v>
       </c>
@@ -4510,11 +3871,11 @@
       <c r="R47" t="s">
         <v>19</v>
       </c>
-      <c r="S47" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="48" spans="1:19">
+      <c r="S47" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>33693</v>
       </c>
@@ -4569,11 +3930,11 @@
       <c r="R48" t="s">
         <v>19</v>
       </c>
-      <c r="S48" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="49" spans="1:19">
+      <c r="S48" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>33693</v>
       </c>
@@ -4628,11 +3989,11 @@
       <c r="R49" t="s">
         <v>19</v>
       </c>
-      <c r="S49" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="50" spans="1:19">
+      <c r="S49" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>33693</v>
       </c>
@@ -4687,11 +4048,11 @@
       <c r="R50" t="s">
         <v>19</v>
       </c>
-      <c r="S50" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="51" spans="1:19">
+      <c r="S50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>33678</v>
       </c>
@@ -4746,11 +4107,11 @@
       <c r="R51" t="s">
         <v>19</v>
       </c>
-      <c r="S51" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="52" spans="1:19">
+      <c r="S51" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>33678</v>
       </c>
@@ -4805,11 +4166,11 @@
       <c r="R52" t="s">
         <v>19</v>
       </c>
-      <c r="S52" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19">
+      <c r="S52" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>33678</v>
       </c>
@@ -4864,11 +4225,11 @@
       <c r="R53" t="s">
         <v>19</v>
       </c>
-      <c r="S53" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19">
+      <c r="S53" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>33678</v>
       </c>
@@ -4923,11 +4284,11 @@
       <c r="R54" t="s">
         <v>19</v>
       </c>
-      <c r="S54" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19">
+      <c r="S54" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>33678</v>
       </c>
@@ -4982,11 +4343,11 @@
       <c r="R55" t="s">
         <v>19</v>
       </c>
-      <c r="S55" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="56" spans="1:19">
+      <c r="S55" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>33678</v>
       </c>
@@ -5041,11 +4402,11 @@
       <c r="R56" t="s">
         <v>19</v>
       </c>
-      <c r="S56" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="57" spans="1:19">
+      <c r="S56" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>33678</v>
       </c>
@@ -5100,11 +4461,11 @@
       <c r="R57" t="s">
         <v>19</v>
       </c>
-      <c r="S57" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="58" spans="1:19">
+      <c r="S57" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>33678</v>
       </c>
@@ -5159,11 +4520,11 @@
       <c r="R58" t="s">
         <v>19</v>
       </c>
-      <c r="S58" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="59" spans="1:19">
+      <c r="S58" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>33678</v>
       </c>
@@ -5218,11 +4579,11 @@
       <c r="R59" t="s">
         <v>19</v>
       </c>
-      <c r="S59" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="60" spans="1:19">
+      <c r="S59" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>33678</v>
       </c>
@@ -5277,11 +4638,11 @@
       <c r="R60" t="s">
         <v>19</v>
       </c>
-      <c r="S60" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19">
+      <c r="S60" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>33678</v>
       </c>
@@ -5336,11 +4697,11 @@
       <c r="R61" t="s">
         <v>19</v>
       </c>
-      <c r="S61" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="62" spans="1:19">
+      <c r="S61" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>33678</v>
       </c>
@@ -5395,11 +4756,11 @@
       <c r="R62" t="s">
         <v>19</v>
       </c>
-      <c r="S62" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="63" spans="1:19">
+      <c r="S62" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>33690</v>
       </c>
@@ -5454,11 +4815,11 @@
       <c r="R63" t="s">
         <v>19</v>
       </c>
-      <c r="S63" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="64" spans="1:19">
+      <c r="S63" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>33690</v>
       </c>
@@ -5513,11 +4874,11 @@
       <c r="R64" t="s">
         <v>19</v>
       </c>
-      <c r="S64" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="65" spans="1:19">
+      <c r="S64" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>33690</v>
       </c>
@@ -5572,11 +4933,11 @@
       <c r="R65" t="s">
         <v>19</v>
       </c>
-      <c r="S65" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="66" spans="1:19">
+      <c r="S65" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>33690</v>
       </c>
@@ -5631,11 +4992,11 @@
       <c r="R66" t="s">
         <v>19</v>
       </c>
-      <c r="S66" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="67" spans="1:19">
+      <c r="S66" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>33690</v>
       </c>
@@ -5690,11 +5051,11 @@
       <c r="R67" t="s">
         <v>19</v>
       </c>
-      <c r="S67" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="68" spans="1:19">
+      <c r="S67" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>33678</v>
       </c>
@@ -5749,11 +5110,11 @@
       <c r="R68" t="s">
         <v>19</v>
       </c>
-      <c r="S68" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="69" spans="1:19">
+      <c r="S68" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>33678</v>
       </c>
@@ -5808,11 +5169,11 @@
       <c r="R69" t="s">
         <v>19</v>
       </c>
-      <c r="S69" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="70" spans="1:19">
+      <c r="S69" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>33678</v>
       </c>
@@ -5867,11 +5228,11 @@
       <c r="R70" t="s">
         <v>19</v>
       </c>
-      <c r="S70" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="71" spans="1:19">
+      <c r="S70" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>33678</v>
       </c>
@@ -5926,11 +5287,11 @@
       <c r="R71" t="s">
         <v>19</v>
       </c>
-      <c r="S71" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="72" spans="1:19">
+      <c r="S71" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>33678</v>
       </c>
@@ -5985,11 +5346,11 @@
       <c r="R72" t="s">
         <v>19</v>
       </c>
-      <c r="S72" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="73" spans="1:19">
+      <c r="S72" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>33678</v>
       </c>
@@ -6044,11 +5405,11 @@
       <c r="R73" t="s">
         <v>19</v>
       </c>
-      <c r="S73" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="74" spans="1:19">
+      <c r="S73" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>33678</v>
       </c>
@@ -6103,11 +5464,11 @@
       <c r="R74" t="s">
         <v>19</v>
       </c>
-      <c r="S74" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="75" spans="1:19">
+      <c r="S74" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>33685</v>
       </c>
@@ -6162,11 +5523,11 @@
       <c r="R75" t="s">
         <v>19</v>
       </c>
-      <c r="S75" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="76" spans="1:19">
+      <c r="S75" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>33692</v>
       </c>
@@ -6221,11 +5582,11 @@
       <c r="R76" t="s">
         <v>19</v>
       </c>
-      <c r="S76" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="77" spans="1:19">
+      <c r="S76" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>33685</v>
       </c>
@@ -6280,11 +5641,11 @@
       <c r="R77" t="s">
         <v>19</v>
       </c>
-      <c r="S77" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="78" spans="1:19">
+      <c r="S77" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>33685</v>
       </c>
@@ -6339,11 +5700,11 @@
       <c r="R78" t="s">
         <v>19</v>
       </c>
-      <c r="S78" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="79" spans="1:19">
+      <c r="S78" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>33692</v>
       </c>
@@ -6398,11 +5759,11 @@
       <c r="R79" t="s">
         <v>19</v>
       </c>
-      <c r="S79" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="80" spans="1:19">
+      <c r="S79" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>33686</v>
       </c>
@@ -6457,11 +5818,11 @@
       <c r="R80" t="s">
         <v>19</v>
       </c>
-      <c r="S80" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="81" spans="1:19">
+      <c r="S80" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>33686</v>
       </c>
@@ -6516,11 +5877,11 @@
       <c r="R81" t="s">
         <v>19</v>
       </c>
-      <c r="S81" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="82" spans="1:19">
+      <c r="S81" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>33686</v>
       </c>
@@ -6575,11 +5936,11 @@
       <c r="R82" t="s">
         <v>19</v>
       </c>
-      <c r="S82" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="83" spans="1:19">
+      <c r="S82" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>33681</v>
       </c>
@@ -6634,11 +5995,11 @@
       <c r="R83" t="s">
         <v>19</v>
       </c>
-      <c r="S83" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="84" spans="1:19">
+      <c r="S83" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>33681</v>
       </c>
@@ -6693,11 +6054,11 @@
       <c r="R84" t="s">
         <v>19</v>
       </c>
-      <c r="S84" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="85" spans="1:19">
+      <c r="S84" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>33681</v>
       </c>
@@ -6752,11 +6113,11 @@
       <c r="R85" t="s">
         <v>19</v>
       </c>
-      <c r="S85" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="86" spans="1:19">
+      <c r="S85" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>33681</v>
       </c>
@@ -6811,11 +6172,11 @@
       <c r="R86" t="s">
         <v>19</v>
       </c>
-      <c r="S86" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="87" spans="1:19">
+      <c r="S86" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>33676</v>
       </c>
@@ -6870,11 +6231,11 @@
       <c r="R87" t="s">
         <v>19</v>
       </c>
-      <c r="S87" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="88" spans="1:19">
+      <c r="S87" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>33700</v>
       </c>
@@ -6929,11 +6290,11 @@
       <c r="R88" t="s">
         <v>19</v>
       </c>
-      <c r="S88" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="89" spans="1:19">
+      <c r="S88" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>33676</v>
       </c>
@@ -6988,11 +6349,11 @@
       <c r="R89" t="s">
         <v>19</v>
       </c>
-      <c r="S89" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="90" spans="1:19">
+      <c r="S89" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>33676</v>
       </c>
@@ -7047,11 +6408,11 @@
       <c r="R90" t="s">
         <v>19</v>
       </c>
-      <c r="S90" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="91" spans="1:19">
+      <c r="S90" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>33700</v>
       </c>
@@ -7106,11 +6467,11 @@
       <c r="R91" t="s">
         <v>19</v>
       </c>
-      <c r="S91" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="92" spans="1:19">
+      <c r="S91" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>33699</v>
       </c>
@@ -7165,11 +6526,11 @@
       <c r="R92" t="s">
         <v>19</v>
       </c>
-      <c r="S92" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="93" spans="1:19">
+      <c r="S92" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>33699</v>
       </c>
@@ -7224,11 +6585,11 @@
       <c r="R93" t="s">
         <v>19</v>
       </c>
-      <c r="S93" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="94" spans="1:19">
+      <c r="S93" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>33699</v>
       </c>
@@ -7283,11 +6644,11 @@
       <c r="R94" t="s">
         <v>19</v>
       </c>
-      <c r="S94" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="95" spans="1:19">
+      <c r="S94" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>19</v>
       </c>
@@ -7346,7 +6707,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" spans="1:19">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>19</v>
       </c>
@@ -7406,103 +6767,7 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="S7" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S2" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S3" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S4" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S5" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S6" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S8" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S9" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S10" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S11" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S12" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S13" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S14" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S15" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S16" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S17" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S18" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S19" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S20" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S21" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S22" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S23" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S24" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S25" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S26" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S27" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S28" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S29" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S30" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S31" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S32" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S33" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S34" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S35" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S36" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S37" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S38" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S39" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S40" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S41" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S42" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S43" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S44" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S45" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S46" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S47" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S48" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S49" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S50" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S51" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S52" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S53" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S54" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S55" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S56" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S57" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S58" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S59" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S60" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S61" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S62" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S63" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S64" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S65" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S66" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S67" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S68" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S69" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S70" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S71" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S72" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S73" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S74" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S75" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S76" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S77" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S78" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S79" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S80" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S81" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S82" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S83" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S84" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S85" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S86" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S87" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S88" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S89" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S90" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S91" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S92" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S93" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-    <hyperlink ref="S94" r:id="rId1" display="alanic.nguetsa@camtrack.net"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>